<commit_message>
Ajusta marcas de escala e remove marcadores da linha no modelo Excel
- Marcas de escala (Tipo Principal) do eixo de categorias passam de
  Cruz para Externo; eixo de valores fica sem marcas, como no padrao
  do R (sem ticks no eixo Y)
- Grafico de linha sem marcadores (bolinhas): somente as linhas
</commit_message>
<xml_diff>
--- a/excel/modelo_graficos_ecoa.xlsx
+++ b/excel/modelo_graficos_ecoa.xlsx
@@ -230,7 +230,7 @@
             </a:ln>
           </c:spPr>
           <c:marker>
-            <c:symbol val="circle"/>
+            <c:symbol val="none"/>
             <c:size val="12"/>
             <c:spPr>
               <a:solidFill>
@@ -387,7 +387,7 @@
             </a:ln>
           </c:spPr>
           <c:marker>
-            <c:symbol val="circle"/>
+            <c:symbol val="none"/>
             <c:size val="12"/>
             <c:spPr>
               <a:solidFill>
@@ -544,7 +544,7 @@
             </a:ln>
           </c:spPr>
           <c:marker>
-            <c:symbol val="circle"/>
+            <c:symbol val="none"/>
             <c:size val="12"/>
             <c:spPr>
               <a:solidFill>
@@ -687,11 +687,11 @@
           <c:showBubbleSize val="0"/>
           <c:separator val=", "/>
         </c:dLbls>
-        <c:axId val="68931999"/>
-        <c:axId val="23847871"/>
+        <c:axId val="22258229"/>
+        <c:axId val="87933916"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="68931999"/>
+        <c:axId val="22258229"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -711,7 +711,7 @@
             </a:ln>
           </c:spPr>
         </c:minorGridlines>
-        <c:majorTickMark val="cross"/>
+        <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
         <c:txPr>
@@ -744,11 +744,11 @@
           </a:ln>
         </c:spPr>
         <c:numFmt formatCode="General" sourceLinked="0"/>
-        <c:crossAx val="23847871"/>
+        <c:crossAx val="87933916"/>
         <c:crosses val="autoZero"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="23847871"/>
+        <c:axId val="87933916"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0.00"/>
@@ -803,7 +803,7 @@
           <c:layout/>
           <c:overlay val="0"/>
         </c:title>
-        <c:majorTickMark val="cross"/>
+        <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
         <c:txPr>
@@ -831,7 +831,7 @@
           </a:ln>
         </c:spPr>
         <c:numFmt formatCode="#,##0" sourceLinked="0"/>
-        <c:crossAx val="68931999"/>
+        <c:crossAx val="22258229"/>
         <c:crosses val="autoZero"/>
       </c:valAx>
       <c:spPr/>
@@ -1105,7 +1105,7 @@
             </a:ln>
           </c:spPr>
         </c:minorGridlines>
-        <c:majorTickMark val="cross"/>
+        <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
         <c:txPr>
@@ -1197,7 +1197,7 @@
           <c:layout/>
           <c:overlay val="0"/>
         </c:title>
-        <c:majorTickMark val="cross"/>
+        <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
         <c:txPr>
@@ -1611,7 +1611,7 @@
             </a:ln>
           </c:spPr>
         </c:minorGridlines>
-        <c:majorTickMark val="cross"/>
+        <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
         <c:txPr>
@@ -1693,7 +1693,7 @@
           <c:layout/>
           <c:overlay val="0"/>
         </c:title>
-        <c:majorTickMark val="cross"/>
+        <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
         <c:txPr>
@@ -2137,7 +2137,7 @@
             </a:ln>
           </c:spPr>
         </c:minorGridlines>
-        <c:majorTickMark val="cross"/>
+        <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
         <c:txPr>
@@ -2229,7 +2229,7 @@
           <c:layout/>
           <c:overlay val="0"/>
         </c:title>
-        <c:majorTickMark val="cross"/>
+        <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
         <c:txPr>

</xml_diff>